<commit_message>
Business case: add Base + incentive column to isolate incentive cost
</commit_message>
<xml_diff>
--- a/business_case.xlsx
+++ b/business_case.xlsx
@@ -261,7 +261,7 @@
     </comment>
     <comment ref="A10" authorId="0" shapeId="0">
       <text>
-        <t>Base design has no price incentive. Low case tests a 30 NTD incentive.</t>
+        <t>Base design has no price incentive. 'Base + incentive' changes only this lever, so it isolates the incentive's cost.</t>
       </text>
     </comment>
   </commentList>
@@ -695,13 +695,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -713,6 +714,7 @@
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -723,12 +725,14 @@
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -748,6 +752,11 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
+          <t>Base + incentive</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
@@ -765,6 +774,9 @@
         <v>0.05</v>
       </c>
       <c r="D5" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E5" s="9" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -781,6 +793,9 @@
         <v>6</v>
       </c>
       <c r="D6" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="10" t="n">
         <v>12</v>
       </c>
     </row>
@@ -797,6 +812,9 @@
         <v>0.3</v>
       </c>
       <c r="D7" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E7" s="9" t="n">
         <v>0.35</v>
       </c>
     </row>
@@ -813,6 +831,9 @@
         <v>2</v>
       </c>
       <c r="D8" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -829,6 +850,9 @@
         <v>0.3</v>
       </c>
       <c r="D9" s="9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E9" s="9" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -845,6 +869,9 @@
         <v>0</v>
       </c>
       <c r="D10" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="E10" s="11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -853,6 +880,7 @@
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -872,6 +900,11 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
+          <t>Base + incentive</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
@@ -894,6 +927,10 @@
         <f>Inputs!$B$5</f>
         <v/>
       </c>
+      <c r="E13" s="12">
+        <f>Inputs!$B$5</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -913,6 +950,10 @@
         <f>D13*D5</f>
         <v/>
       </c>
+      <c r="E14" s="13">
+        <f>E13*E5</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -932,6 +973,10 @@
         <f>D14*Inputs!$B$7*D7*D6</f>
         <v/>
       </c>
+      <c r="E15" s="14">
+        <f>E14*Inputs!$B$7*E7*E6</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -951,6 +996,10 @@
         <f>D13*D8+D13*D9*D10</f>
         <v/>
       </c>
+      <c r="E16" s="14">
+        <f>E13*E8+E13*E9*E10</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
@@ -970,6 +1019,10 @@
         <f>D15-D16</f>
         <v/>
       </c>
+      <c r="E17" s="16">
+        <f>E15-E16</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -989,6 +1042,10 @@
         <f>IFERROR(D17/D16,"n/a")</f>
         <v/>
       </c>
+      <c r="E18" s="17">
+        <f>IFERROR(E17/E16,"n/a")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
@@ -1008,6 +1065,10 @@
         <f>IFERROR(D16/(D13*Inputs!$B$7*D7*D6),0)</f>
         <v/>
       </c>
+      <c r="E19" s="18">
+        <f>IFERROR(E16/(E13*Inputs!$B$7*E7*E6),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1025,6 +1086,10 @@
       </c>
       <c r="D20" s="5">
         <f>IF(D5&gt;=D19,"Above break-even","Below break-even")</f>
+        <v/>
+      </c>
+      <c r="E20" s="5">
+        <f>IF(E5&gt;=E19,"Above break-even","Below break-even")</f>
         <v/>
       </c>
     </row>
@@ -1033,6 +1098,7 @@
       <c r="B21" s="2" t="n"/>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
@@ -1043,6 +1109,7 @@
       <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1057,6 +1124,7 @@
       </c>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -1068,6 +1136,7 @@
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -1079,6 +1148,7 @@
       </c>
       <c r="C25" s="2" t="n"/>
       <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -1090,6 +1160,7 @@
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -1101,6 +1172,7 @@
       </c>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -1112,6 +1184,7 @@
       </c>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -1123,12 +1196,14 @@
       </c>
       <c r="C29" s="2" t="n"/>
       <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n"/>
       <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1139,6 +1214,18 @@
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="n"/>
       <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>'Base + incentive' equals Base except for a 30 NTD incentive per opt-in. It shows how much extra churn reduction an incentive must buy just to pay for itself.</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1431,7 +1518,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Opt-in rate, incentive</t>
+          <t>Opt-in rate, 30 NTD incentive</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1446,7 +1533,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Only matters with an incentive</t>
+          <t>Incentive needs about 4.3 points to break even</t>
         </is>
       </c>
     </row>

</xml_diff>